<commit_message>
chore(report): refresh xlsx template with gateway quota rows
Mirrors the new Section 9 (LLM) and Section 6 (OCR/VLM) added in the
parent repo's llm_calc/ocr_calc generators.
</commit_message>
<xml_diff>
--- a/backend/reportTemplate.xlsx
+++ b/backend/reportTemplate.xlsx
@@ -250,10 +250,10 @@
     <xf numFmtId="11" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3307,7 +3307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -5219,112 +5219,286 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>9. Квоты для шлюза (LiteLLM / shared vLLM)</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="n"/>
+      <c r="C75" s="6" t="n"/>
+      <c r="D75" s="6" t="n"/>
+      <c r="E75" s="6" t="n"/>
+      <c r="F75" s="7" t="n"/>
+    </row>
     <row r="76">
-      <c r="A76" s="5" t="inlineStr">
+      <c r="A76" s="8" t="inlineStr">
+        <is>
+          <t>Peak RPM (запросов/мин с headroom)</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>S_sim · R · K_SLA · 60 — пиковый RPM для конфигурации шлюза</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>calc</t>
+        </is>
+      </c>
+      <c r="D76" s="25">
+        <f>Inputs!D12*Inputs!D75*Inputs!D76*60</f>
+        <v/>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>req/min</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>🔵 derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
+          <t>Sustained RPM (без headroom)</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>S_sim · R · 60 — устоявшийся RPM</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>calc</t>
+        </is>
+      </c>
+      <c r="D77" s="25">
+        <f>Inputs!D12*Inputs!D75*60</f>
+        <v/>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>req/min</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>🔵 derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t>Peak TPM input</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>peak_rpm · SL_pf — input-side tokens/min</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>calc</t>
+        </is>
+      </c>
+      <c r="D78" s="25">
+        <f>D76*Inputs!D21</f>
+        <v/>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>tok/min</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>🔵 derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="inlineStr">
+        <is>
+          <t>Peak TPM output</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>peak_rpm · T_dec — output-side tokens/min</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>calc</t>
+        </is>
+      </c>
+      <c r="D79" s="25">
+        <f>D76*Inputs!D22</f>
+        <v/>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>tok/min</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>🔵 derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>Peak TPM (total)</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>peak_tpm_input + peak_tpm_output</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>calc</t>
+        </is>
+      </c>
+      <c r="D80" s="25">
+        <f>D78+D79</f>
+        <v/>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>tok/min</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>🔵 derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="8" t="inlineStr">
+        <is>
+          <t>Sustained TPM (без headroom)</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>peak_tpm / K_SLA</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>calc</t>
+        </is>
+      </c>
+      <c r="D81" s="25">
+        <f>IF(Inputs!D76&gt;0,D80/Inputs!D76,D80)</f>
+        <v/>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>tok/min</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>🔵 derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>Max parallel requests</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>⌈S_sim · K_SLA⌉ — лимит конкурентных запросов</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>calc</t>
+        </is>
+      </c>
+      <c r="D82" s="17">
+        <f>CEILING(Inputs!D12*Inputs!D76,1)</f>
+        <v/>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>req</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>🔵 derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
         <is>
           <t>📋 Валидация расчётных значений на реальном оборудовании</t>
         </is>
       </c>
-      <c r="B76" s="6" t="n"/>
-      <c r="C76" s="6" t="n"/>
-      <c r="D76" s="6" t="n"/>
-      <c r="E76" s="6" t="n"/>
-      <c r="F76" s="7" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>Колонка «F» рядом с каждым значением показывает, КАК проверить число на реальной системе:</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟢 EvalScope       — получено из нагрузочного теста (см. инструкции ниже)</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟢 deployment      — проверяется при фактическом развёртывании (vLLM/SGLang)</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟡 vLLM logs       — видно в логах инференс-движка (--log-stats)</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🟡 nvidia-smi      — проверяется через nvidia-smi / dcgm</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ⚪ derived / methodology / spec lookup — производные величины, не проверяются эмпирически</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="4" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="4" t="inlineStr">
-        <is>
-          <t>🔬 Процедура валидации через EvalScope (Прил. Е методологии):</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="4" t="inlineStr"/>
+      <c r="B85" s="6" t="n"/>
+      <c r="C85" s="6" t="n"/>
+      <c r="D85" s="6" t="n"/>
+      <c r="E85" s="6" t="n"/>
+      <c r="F85" s="7" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>ШАГ 1. Decode-heavy прогон (калибровка η_mem, см. §Е.1.1):</t>
+          <t>Колонка «F» рядом с каждым значением показывает, КАК проверить число на реальной системе:</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  evalscope perf --url http://localhost:8000/v1/chat/completions \</t>
+          <t xml:space="preserve">  🟢 EvalScope       — получено из нагрузочного теста (см. инструкции ниже)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">       --parallel 30  --number 30  --min-tokens 1000  --max-tokens 1000 \</t>
+          <t xml:space="preserve">  🟢 deployment      — проверяется при фактическом развёртывании (vLLM/SGLang)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">       --min-prompt-length 400  --max-prompt-length 600  --dataset random</t>
+          <t xml:space="preserve">  🟡 vLLM logs       — видно в логах инференс-движка (--log-stats)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Снимаемая метрика: Th_dec_observed = Output token throughput (tok/s, серверный агрегат).</t>
+          <t xml:space="preserve">  🟡 nvidia-smi      — проверяется через nvidia-smi / dcgm</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Сравнить с ячейкой «Th_dec (per-session)» × BS × N_TP=Z. Расхождение &gt;20% → пересчитать η_mem (§Е.2).</t>
+          <t xml:space="preserve">  ⚪ derived / methodology / spec lookup — производные величины, не проверяются эмпирически</t>
         </is>
       </c>
     </row>
@@ -5334,134 +5508,190 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>ШАГ 2. Prefill-heavy прогон (калибровка η_pf, см. §Е.1.2):</t>
+          <t>🔬 Процедура валидации через EvalScope (Прил. Е методологии):</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  evalscope perf --url http://localhost:8000/v1/chat/completions \</t>
-        </is>
-      </c>
+      <c r="A94" s="4" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">       --parallel 30  --number 30  --min-tokens 1  --max-tokens 1 \</t>
+          <t>ШАГ 1. Decode-heavy прогон (калибровка η_mem, см. §Е.1.1):</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">       --min-prompt-length 7000  --max-prompt-length 9000  --dataset random</t>
+          <t xml:space="preserve">  evalscope perf --url http://localhost:8000/v1/chat/completions \</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Снимаемая метрика: Th_pf_observed = (Total throughput − Output throughput).</t>
+          <t xml:space="preserve">       --parallel 30  --number 30  --min-tokens 1000  --max-tokens 1000 \</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Сравнить с ячейкой «Th_pf (per-session)» × BS × N_TP=Z. Расхождение &gt;20% → пересчитать η_pf (§Е.3).</t>
+          <t xml:space="preserve">       --min-prompt-length 400  --max-prompt-length 600  --dataset random</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="4" t="inlineStr"/>
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Снимаемая метрика: Th_dec_observed = Output token throughput (tok/s, серверный агрегат).</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>ШАГ 3. Проверка по закону Литтла (§Е.4):</t>
+          <t xml:space="preserve">  Сравнить с ячейкой «Th_dec (per-session)» × BS × N_TP=Z. Расхождение &gt;20% → пересчитать η_mem (§Е.2).</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Должно выполняться: BS ≈ λ · W_mean (где λ — RPS, W_mean — средняя end-to-end задержка).</t>
-        </is>
-      </c>
+      <c r="A101" s="4" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Погрешность &gt;10% указывает на некорректную постановку теста.</t>
+          <t>ШАГ 2. Prefill-heavy прогон (калибровка η_pf, см. §Е.1.2):</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="4" t="inlineStr"/>
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  evalscope perf --url http://localhost:8000/v1/chat/completions \</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>ШАГ 4. Если η_mem или η_pf отличаются от дефолтов — ввести откалиброванные значения</t>
+          <t xml:space="preserve">       --parallel 30  --number 30  --min-tokens 1  --max-tokens 1 \</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  в Inputs!η_mem и Inputs!η_pf, пересчитать Sizing. Затем повторить Шаги 1–2 для валидации.</t>
+          <t xml:space="preserve">       --min-prompt-length 7000  --max-prompt-length 9000  --dataset random</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="4" t="inlineStr"/>
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Снимаемая метрика: Th_pf_observed = (Total throughput − Output throughput).</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>Альтернативы EvalScope (эквивалентная методика, см. Прил. Е.8):</t>
+          <t xml:space="preserve">  Сравнить с ячейкой «Th_pf (per-session)» × BS × N_TP=Z. Расхождение &gt;20% → пересчитать η_pf (§Е.3).</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • NVIDIA GenAI-Perf (для NIM/TensorRT-LLM эндпоинтов)</t>
-        </is>
-      </c>
+      <c r="A108" s="4" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • vllm_benchmarks/benchmark_serving.py (из репозитория vllm-project/vllm)</t>
+          <t>ШАГ 3. Проверка по закону Литтла (§Е.4):</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Должно выполняться: BS ≈ λ · W_mean (где λ — RPS, W_mean — средняя end-to-end задержка).</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Погрешность &gt;10% указывает на некорректную постановку теста.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="4" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="4" t="inlineStr">
+        <is>
+          <t>ШАГ 4. Если η_mem или η_pf отличаются от дефолтов — ввести откалиброванные значения</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  в Inputs!η_mem и Inputs!η_pf, пересчитать Sizing. Затем повторить Шаги 1–2 для валидации.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>Альтернативы EvalScope (эквивалентная методика, см. Прил. Е.8):</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • NVIDIA GenAI-Perf (для NIM/TensorRT-LLM эндпоинтов)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • vllm_benchmarks/benchmark_serving.py (из репозитория vllm-project/vllm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • sglang/bench_serving.py (из репозитория sgl-project/sglang)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="43">
+  <mergeCells count="44">
     <mergeCell ref="A99:F99"/>
-    <mergeCell ref="A84:F84"/>
     <mergeCell ref="A90:F90"/>
+    <mergeCell ref="A108:F108"/>
     <mergeCell ref="A66:F66"/>
-    <mergeCell ref="A108:F108"/>
-    <mergeCell ref="A80:F80"/>
+    <mergeCell ref="A118:F118"/>
+    <mergeCell ref="A75:F75"/>
     <mergeCell ref="A89:F89"/>
     <mergeCell ref="A105:F105"/>
     <mergeCell ref="A101:F101"/>
     <mergeCell ref="A86:F86"/>
     <mergeCell ref="A104:F104"/>
     <mergeCell ref="A95:F95"/>
+    <mergeCell ref="A113:F113"/>
     <mergeCell ref="A85:F85"/>
     <mergeCell ref="A42:F42"/>
-    <mergeCell ref="A76:F76"/>
+    <mergeCell ref="A116:F116"/>
     <mergeCell ref="A106:F106"/>
     <mergeCell ref="A97:F97"/>
     <mergeCell ref="A4:F4"/>
@@ -5470,25 +5700,25 @@
     <mergeCell ref="A96:F96"/>
     <mergeCell ref="A91:F91"/>
     <mergeCell ref="A109:F109"/>
-    <mergeCell ref="A81:F81"/>
+    <mergeCell ref="A115:F115"/>
+    <mergeCell ref="A112:F112"/>
     <mergeCell ref="A93:F93"/>
     <mergeCell ref="A102:F102"/>
+    <mergeCell ref="A117:F117"/>
     <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A111:F111"/>
     <mergeCell ref="A58:F58"/>
-    <mergeCell ref="A83:F83"/>
     <mergeCell ref="A92:F92"/>
-    <mergeCell ref="A77:F77"/>
+    <mergeCell ref="A114:F114"/>
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A107:F107"/>
-    <mergeCell ref="A82:F82"/>
     <mergeCell ref="A98:F98"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A94:F94"/>
     <mergeCell ref="A103:F103"/>
-    <mergeCell ref="A79:F79"/>
     <mergeCell ref="A110:F110"/>
+    <mergeCell ref="A119:F119"/>
     <mergeCell ref="A88:F88"/>
-    <mergeCell ref="A78:F78"/>
     <mergeCell ref="A87:F87"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:D2000">
@@ -6127,7 +6357,7 @@
           <t>calc</t>
         </is>
       </c>
-      <c r="D43" s="25">
+      <c r="D43" s="26">
         <f>Inputs!D75*D23</f>
         <v/>
       </c>
@@ -6867,7 +7097,7 @@
           <t>calc</t>
         </is>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="25">
         <f>IF(AND(D7&gt;0,Inputs!D28&gt;0),D8*(IF(Inputs!D52,(Inputs!D48+Inputs!D49*(1-POWER(1-Inputs!D50/Inputs!D51,D7))),Inputs!D37)*10^9*Inputs!D54+D7*D11*1024^3)/(Inputs!D28*10^9*D7*Sizing!D12),0)</f>
         <v/>
       </c>
@@ -6893,7 +7123,7 @@
           <t>calc</t>
         </is>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="25">
         <f>IF(AND(Sizing!D26&gt;0,D7&gt;0,Sizing!D12&gt;0),D8*(Sizing!D25+4*Inputs!D38*Inputs!D39*(D9+(D10-1)/2))*D7/(Sizing!D26*Sizing!D12),0)</f>
         <v/>
       </c>
@@ -7113,7 +7343,7 @@
           <t>calc</t>
         </is>
       </c>
-      <c r="D24" s="26">
+      <c r="D24" s="25">
         <f>IF(ABS(D22-D23)&gt;0.01,(D23*D21-D22*D20)/(1024^3*(D22-D23)),0)</f>
         <v/>
       </c>
@@ -7139,7 +7369,7 @@
           <t>calc</t>
         </is>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="25">
         <f>IF(AND(D22&gt;0,Inputs!D28&gt;0),D22*(D20+D24*1024^3)/(Inputs!D28*10^9),0)</f>
         <v/>
       </c>
@@ -7252,7 +7482,7 @@
           <t>calc</t>
         </is>
       </c>
-      <c r="D31" s="26">
+      <c r="D31" s="25">
         <f>IF(AND(Sizing!D26&gt;0,D7&gt;0,Sizing!D12&gt;0),D29*(Sizing!D25+4*Inputs!D38*Inputs!D39*D30)/(Sizing!D26*D7*Sizing!D12),0)</f>
         <v/>
       </c>
@@ -8562,16 +8792,16 @@
         <v>0</v>
       </c>
       <c r="M34" s="29" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="N34" s="29" t="n">
-        <v>32.5</v>
+        <v>0</v>
       </c>
       <c r="O34" s="29" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P34" s="29" t="n">
-        <v>128</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">

</xml_diff>